<commit_message>
data(swarm-disaster): G09-P4-B2 execute semantic fixtures
</commit_message>
<xml_diff>
--- a/config/swarm-disaster-generated/templates/SwarmDisasterEvidence.xlsx
+++ b/config/swarm-disaster-generated/templates/SwarmDisasterEvidence.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="914" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="934" uniqueCount="155">
   <si>
     <t>@table</t>
   </si>
@@ -264,7 +264,7 @@
     <t>SwarmDisasterResearchGap</t>
   </si>
   <si>
-    <t>c053f179e53b4d47</t>
+    <t>89be6c0263ec2ed2</t>
   </si>
   <si>
     <t>state</t>
@@ -288,6 +288,18 @@
     <t>selected_policy</t>
   </si>
   <si>
+    <t>rejected_alternatives</t>
+  </si>
+  <si>
+    <t>rationale</t>
+  </si>
+  <si>
+    <t>affected_fixture_ids</t>
+  </si>
+  <si>
+    <t>confidence</t>
+  </si>
+  <si>
     <t>bool</t>
   </si>
   <si>
@@ -295,6 +307,12 @@
   </si>
   <si>
     <t>length=1..4000</t>
+  </si>
+  <si>
+    <t>parser=split;separator=|;length=1..4</t>
+  </si>
+  <si>
+    <t>parser=split;separator=|;length=1..16</t>
   </si>
   <si>
     <t>SwarmDisasterResearchGapAffected</t>
@@ -2057,7 +2075,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W7"/>
+  <dimension ref="A1:AA7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -2072,11 +2090,14 @@
     <col min="19" max="19" width="16.7109375" style="5" customWidth="1"/>
     <col min="20" max="20" width="12.7109375" style="5" customWidth="1"/>
     <col min="21" max="21" width="15.7109375" style="5" customWidth="1"/>
-    <col min="22" max="22" width="12.7109375" style="5" customWidth="1"/>
-    <col min="23" max="23" width="21.7109375" style="5" customWidth="1"/>
+    <col min="22" max="22" width="21.7109375" style="5" customWidth="1"/>
+    <col min="23" max="23" width="12.7109375" style="5" customWidth="1"/>
+    <col min="24" max="24" width="20.7109375" style="5" customWidth="1"/>
+    <col min="25" max="26" width="12.7109375" style="5" customWidth="1"/>
+    <col min="27" max="27" width="21.7109375" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23">
+    <row r="1" spans="1:27">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2108,7 +2129,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="2" spans="1:23" ht="24" customHeight="1">
+    <row r="2" spans="1:27" ht="24" customHeight="1">
       <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
@@ -2173,13 +2194,25 @@
         <v>87</v>
       </c>
       <c r="V2" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="W2" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="X2" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="Y2" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="Z2" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="W2" s="3" t="s">
+      <c r="AA2" s="3" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="3" spans="1:23">
+    <row r="3" spans="1:27">
       <c r="A3" s="4" t="s">
         <v>31</v>
       </c>
@@ -2244,13 +2277,25 @@
         <v>87</v>
       </c>
       <c r="V3" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="Y3" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="Z3" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="W3" s="5" t="s">
+      <c r="AA3" s="5" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:23">
+    <row r="4" spans="1:27">
       <c r="A4" s="4" t="s">
         <v>32</v>
       </c>
@@ -2300,7 +2345,7 @@
         <v>34</v>
       </c>
       <c r="Q4" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="R4" s="5" t="s">
         <v>34</v>
@@ -2315,13 +2360,25 @@
         <v>34</v>
       </c>
       <c r="V4" s="5" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="W4" s="5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="5" spans="1:23">
+      <c r="X4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Y4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="Z4" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="AA4" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:27">
       <c r="A5" s="4" t="s">
         <v>41</v>
       </c>
@@ -2391,8 +2448,20 @@
       <c r="W5" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:23">
+      <c r="X5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Y5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="Z5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="AA5" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27">
       <c r="A6" s="4" t="s">
         <v>42</v>
       </c>
@@ -2430,10 +2499,10 @@
         <v>48</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="Q6" s="5"/>
       <c r="R6" s="5" t="s">
@@ -2443,19 +2512,31 @@
         <v>44</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="V6" s="5" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="W6" s="5" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" ht="42" customHeight="1">
+        <v>94</v>
+      </c>
+      <c r="X6" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="Y6" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="Z6" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="AA6" s="5" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" ht="42" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>53</v>
       </c>
@@ -2481,6 +2562,10 @@
       <c r="U7" s="6"/>
       <c r="V7" s="6"/>
       <c r="W7" s="6"/>
+      <c r="X7" s="6"/>
+      <c r="Y7" s="6"/>
+      <c r="Z7" s="6"/>
+      <c r="AA7" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="5">
@@ -2522,7 +2607,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2546,7 +2631,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -2557,16 +2642,16 @@
         <v>5</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -2577,16 +2662,16 @@
         <v>5</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -2597,7 +2682,7 @@
         <v>33</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>33</v>
@@ -2638,7 +2723,7 @@
       </c>
       <c r="C6" s="5"/>
       <c r="D6" s="5" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>44</v>
@@ -2702,7 +2787,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -2726,7 +2811,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:24" ht="24" customHeight="1">
@@ -2776,25 +2861,25 @@
         <v>23</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="W2" s="3" t="s">
         <v>65</v>
@@ -2850,25 +2935,25 @@
         <v>23</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="W3" s="5" t="s">
         <v>65</v>
@@ -3066,7 +3151,7 @@
         <v>49</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>51</v>
@@ -3081,7 +3166,7 @@
         <v>51</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="V6" s="5"/>
       <c r="W6" s="5"/>
@@ -3165,7 +3250,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3189,7 +3274,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="24" customHeight="1">
@@ -3236,31 +3321,31 @@
         <v>22</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:23">
@@ -3307,31 +3392,31 @@
         <v>22</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" spans="1:23">
@@ -3622,7 +3707,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -3646,7 +3731,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2" spans="1:24" ht="24" customHeight="1">
@@ -3663,64 +3748,64 @@
         <v>12</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:24">
@@ -3737,64 +3822,64 @@
         <v>12</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="Q3" s="5" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="R3" s="5" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="S3" s="5" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="T3" s="5" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="V3" s="5" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="W3" s="5" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="X3" s="5" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:24">
@@ -3865,7 +3950,7 @@
         <v>34</v>
       </c>
       <c r="W4" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="X4" s="5" t="s">
         <v>39</v>
@@ -3950,7 +4035,7 @@
         <v>42</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>44</v>
@@ -3980,31 +4065,31 @@
         <v>70</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="M6" s="5" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="N6" s="5" t="s">
         <v>69</v>
       </c>
       <c r="O6" s="5" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="P6" s="5" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="Q6" s="5" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="R6" s="5" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="S6" s="5" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="T6" s="5" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="U6" s="5" t="s">
         <v>45</v>
@@ -4014,7 +4099,7 @@
       </c>
       <c r="W6" s="5"/>
       <c r="X6" s="5" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
     </row>
     <row r="7" spans="1:24" ht="42" customHeight="1">
@@ -4107,7 +4192,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
@@ -4131,7 +4216,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="24" customHeight="1">
@@ -4148,19 +4233,19 @@
         <v>12</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>63</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -4177,19 +4262,19 @@
         <v>12</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>63</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -4267,10 +4352,10 @@
         <v>44</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>70</v>

</xml_diff>